<commit_message>
feat: final video list (all verified)
</commit_message>
<xml_diff>
--- a/videos.xlsx
+++ b/videos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Alex\Documents\GitHub\ro-av-deepfake-dataset\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13DBC9F5-4546-4863-8898-10CFF4534117}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB3E3681-020B-4BBC-BF0D-BEF8907F6E8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Muntenia" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1199" uniqueCount="540">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1200" uniqueCount="543">
   <si>
     <t>https://www.youtube.com/watch?v=l2I7D1HsJmw</t>
   </si>
@@ -1224,9 +1224,6 @@
     <t>https://www.youtube.com/watch?v=JPjXgv8mzIY</t>
   </si>
   <si>
-    <t>https://www.youtube.com/watch?v=IIA2y625iuY</t>
-  </si>
-  <si>
     <t>https://www.youtube.com/watch?v=c-SOl7TYoNs</t>
   </si>
   <si>
@@ -1296,9 +1293,6 @@
     <t>0:00-3:51</t>
   </si>
   <si>
-    <t>https://www.youtube.com/watch?v=e8r-1M5V4Yo</t>
-  </si>
-  <si>
     <t>https://www.youtube.com/watch?v=Wonhi3yRu5c</t>
   </si>
   <si>
@@ -1660,6 +1654,21 @@
   </si>
   <si>
     <t>0:00-6:46</t>
+  </si>
+  <si>
+    <t>0:00-7:05</t>
+  </si>
+  <si>
+    <t>0:00-5:52</t>
+  </si>
+  <si>
+    <t>0:00-5:15</t>
+  </si>
+  <si>
+    <t>4:32-7:45</t>
+  </si>
+  <si>
+    <t>2:19-7:31</t>
   </si>
 </sst>
 </file>
@@ -1739,7 +1748,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1756,7 +1765,6 @@
     <xf numFmtId="20" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="2"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="2" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2077,10 +2085,10 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{5FB8BC92-48E7-4C5E-8055-292233253902}" name="Table5" displayName="Table5" ref="A1:E87" totalsRowShown="0" headerRowDxfId="25" dataDxfId="24" tableBorderDxfId="23" headerRowCellStyle="Output">
-  <autoFilter ref="A1:E87" xr:uid="{5FB8BC92-48E7-4C5E-8055-292233253902}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:E87">
-    <sortCondition descending="1" ref="D1:D87"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{5FB8BC92-48E7-4C5E-8055-292233253902}" name="Table5" displayName="Table5" ref="A1:E85" totalsRowShown="0" headerRowDxfId="25" dataDxfId="24" tableBorderDxfId="23" headerRowCellStyle="Output">
+  <autoFilter ref="A1:E85" xr:uid="{5FB8BC92-48E7-4C5E-8055-292233253902}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:E85">
+    <sortCondition descending="1" ref="D1:D85"/>
   </sortState>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{E853F3B6-335F-4CE8-AA32-003A4EFDCCA1}" name="Link" dataDxfId="22"/>
@@ -2401,20 +2409,20 @@
     <col min="6" max="6" width="20.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="9" t="s">
+    <row r="1" spans="1:5" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="8" t="s">
         <v>73</v>
       </c>
-      <c r="B1" s="10" t="s">
+      <c r="B1" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="C1" s="9" t="s">
+      <c r="C1" s="8" t="s">
         <v>111</v>
       </c>
-      <c r="D1" s="10" t="s">
+      <c r="D1" s="9" t="s">
         <v>74</v>
       </c>
-      <c r="E1" s="10" t="s">
+      <c r="E1" s="9" t="s">
         <v>75</v>
       </c>
     </row>
@@ -2526,7 +2534,7 @@
         <v>4</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>533</v>
+        <v>531</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
@@ -2543,7 +2551,7 @@
         <v>4</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
@@ -2560,7 +2568,7 @@
         <v>4</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>535</v>
+        <v>533</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
@@ -2577,7 +2585,7 @@
         <v>4</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>536</v>
+        <v>534</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
@@ -2730,7 +2738,7 @@
         <v>4</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>532</v>
+        <v>530</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
@@ -2747,7 +2755,7 @@
         <v>4</v>
       </c>
       <c r="E21" s="5" t="s">
-        <v>531</v>
+        <v>529</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
@@ -2764,7 +2772,7 @@
         <v>4</v>
       </c>
       <c r="E22" s="5" t="s">
-        <v>530</v>
+        <v>528</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
@@ -2781,7 +2789,7 @@
         <v>4</v>
       </c>
       <c r="E23" s="5" t="s">
-        <v>529</v>
+        <v>527</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
@@ -2798,7 +2806,7 @@
         <v>4</v>
       </c>
       <c r="E24" s="5" t="s">
-        <v>528</v>
+        <v>526</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
@@ -2815,7 +2823,7 @@
         <v>4</v>
       </c>
       <c r="E25" s="5" t="s">
-        <v>527</v>
+        <v>525</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
@@ -2832,7 +2840,7 @@
         <v>4</v>
       </c>
       <c r="E26" s="5" t="s">
-        <v>526</v>
+        <v>524</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
@@ -2849,7 +2857,7 @@
         <v>4</v>
       </c>
       <c r="E27" s="5" t="s">
-        <v>525</v>
+        <v>523</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
@@ -3271,7 +3279,7 @@
         <v>4</v>
       </c>
       <c r="E53" s="5" t="s">
-        <v>524</v>
+        <v>522</v>
       </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.25">
@@ -3825,7 +3833,7 @@
         <v>2</v>
       </c>
       <c r="E89" s="5" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.25">
@@ -3932,7 +3940,7 @@
         <v>1</v>
       </c>
       <c r="C96" s="2" t="s">
-        <v>522</v>
+        <v>520</v>
       </c>
       <c r="D96" s="5" t="s">
         <v>2</v>
@@ -4056,20 +4064,20 @@
     <col min="5" max="5" width="20.85546875" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="9" t="s">
+    <row r="1" spans="1:5" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="8" t="s">
         <v>73</v>
       </c>
-      <c r="B1" s="10" t="s">
+      <c r="B1" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="C1" s="9" t="s">
+      <c r="C1" s="8" t="s">
         <v>111</v>
       </c>
-      <c r="D1" s="10" t="s">
+      <c r="D1" s="9" t="s">
         <v>74</v>
       </c>
-      <c r="E1" s="10" t="s">
+      <c r="E1" s="9" t="s">
         <v>75</v>
       </c>
     </row>
@@ -4192,7 +4200,7 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>473</v>
+        <v>471</v>
       </c>
       <c r="B9" s="5">
         <v>1</v>
@@ -4209,7 +4217,7 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>474</v>
+        <v>472</v>
       </c>
       <c r="B10" s="5">
         <v>1</v>
@@ -4226,7 +4234,7 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>475</v>
+        <v>473</v>
       </c>
       <c r="B11" s="5">
         <v>1</v>
@@ -4238,7 +4246,7 @@
         <v>4</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>476</v>
+        <v>474</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
@@ -4406,7 +4414,7 @@
         <v>4</v>
       </c>
       <c r="E21" s="5" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
@@ -4426,7 +4434,7 @@
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
-        <v>466</v>
+        <v>464</v>
       </c>
       <c r="B23" s="5">
         <v>1</v>
@@ -4438,12 +4446,12 @@
         <v>4</v>
       </c>
       <c r="E23" s="5" t="s">
-        <v>467</v>
+        <v>465</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
-        <v>468</v>
+        <v>466</v>
       </c>
       <c r="B24" s="5">
         <v>1</v>
@@ -4458,7 +4466,7 @@
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
-        <v>471</v>
+        <v>469</v>
       </c>
       <c r="B25" s="5">
         <v>1</v>
@@ -4470,7 +4478,7 @@
         <v>4</v>
       </c>
       <c r="E25" s="5" t="s">
-        <v>472</v>
+        <v>470</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
@@ -4773,7 +4781,7 @@
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" s="3" t="s">
-        <v>463</v>
+        <v>461</v>
       </c>
       <c r="B44" s="5">
         <v>1</v>
@@ -4785,7 +4793,7 @@
         <v>4</v>
       </c>
       <c r="E44" s="5" t="s">
-        <v>464</v>
+        <v>462</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.25">
@@ -4853,7 +4861,7 @@
         <v>2</v>
       </c>
       <c r="E48" s="5" t="s">
-        <v>537</v>
+        <v>535</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.25">
@@ -4930,7 +4938,7 @@
         <v>2</v>
       </c>
       <c r="E53" s="5" t="s">
-        <v>538</v>
+        <v>536</v>
       </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.25">
@@ -5012,7 +5020,7 @@
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A59" s="3" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="B59" s="5">
         <v>1</v>
@@ -5024,7 +5032,7 @@
         <v>2</v>
       </c>
       <c r="E59" s="5" t="s">
-        <v>478</v>
+        <v>476</v>
       </c>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.25">
@@ -5071,7 +5079,7 @@
         <v>2</v>
       </c>
       <c r="E62" s="5" t="s">
-        <v>539</v>
+        <v>537</v>
       </c>
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.25">
@@ -5223,7 +5231,7 @@
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A72" s="3" t="s">
-        <v>469</v>
+        <v>467</v>
       </c>
       <c r="B72" s="5">
         <v>1</v>
@@ -5238,7 +5246,7 @@
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A73" s="3" t="s">
-        <v>470</v>
+        <v>468</v>
       </c>
       <c r="B73" s="5">
         <v>1</v>
@@ -5481,7 +5489,7 @@
     </row>
     <row r="88" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A88" s="3" t="s">
-        <v>512</v>
+        <v>510</v>
       </c>
       <c r="B88" s="5">
         <v>1</v>
@@ -5593,7 +5601,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8D66C23E-87E5-4813-AF0A-DC21A95E91BE}">
-  <dimension ref="A1:E78"/>
+  <dimension ref="A1:E76"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="69" customWidth="1"/>
@@ -5603,37 +5611,41 @@
     <col min="5" max="5" width="20.140625" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="9" t="s">
+    <row r="1" spans="1:5" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="8" t="s">
         <v>73</v>
       </c>
-      <c r="B1" s="10" t="s">
+      <c r="B1" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="C1" s="9" t="s">
+      <c r="C1" s="8" t="s">
         <v>111</v>
       </c>
-      <c r="D1" s="10" t="s">
+      <c r="D1" s="9" t="s">
         <v>74</v>
       </c>
-      <c r="E1" s="10" t="s">
+      <c r="E1" s="9" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="8" t="s">
+      <c r="A2" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C2" t="s">
+      <c r="B2" s="5"/>
+      <c r="C2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="1" t="s">
-        <v>4</v>
+      <c r="D2" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>542</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="B3" s="5">
         <v>1</v>
@@ -5645,12 +5657,12 @@
         <v>4</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="B4" s="5">
         <v>1</v>
@@ -5662,12 +5674,12 @@
         <v>4</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="B5" s="5">
         <v>1</v>
@@ -5679,12 +5691,12 @@
         <v>4</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="B6" s="5">
         <v>1</v>
@@ -5696,56 +5708,57 @@
         <v>4</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>458</v>
+        <v>456</v>
       </c>
       <c r="B7" s="5">
         <v>1</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>454</v>
+        <v>452</v>
       </c>
       <c r="D7" s="5" t="s">
         <v>4</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>459</v>
+        <v>457</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>460</v>
+        <v>458</v>
       </c>
       <c r="B8" s="5">
         <v>1</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>454</v>
+        <v>452</v>
       </c>
       <c r="D8" s="5" t="s">
         <v>4</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>461</v>
+        <v>459</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" s="8" t="s">
-        <v>465</v>
-      </c>
-      <c r="B9" s="1">
-        <v>1</v>
-      </c>
-      <c r="C9" t="s">
-        <v>454</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>4</v>
-      </c>
+      <c r="A9" s="3" t="s">
+        <v>463</v>
+      </c>
+      <c r="B9" s="5">
+        <v>1</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>452</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="E9" s="5"/>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
@@ -5765,131 +5778,157 @@
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" s="8" t="s">
+      <c r="A11" s="3" t="s">
         <v>393</v>
       </c>
-      <c r="B11" s="1">
-        <v>1</v>
-      </c>
-      <c r="C11" t="s">
+      <c r="B11" s="5">
+        <v>1</v>
+      </c>
+      <c r="C11" s="2" t="s">
         <v>389</v>
       </c>
-      <c r="D11" s="1" t="s">
-        <v>4</v>
-      </c>
+      <c r="D11" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="E11" s="5"/>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" s="8" t="s">
-        <v>394</v>
-      </c>
-      <c r="B12" s="1">
-        <v>1</v>
-      </c>
-      <c r="C12" t="s">
+      <c r="A12" s="3" t="s">
+        <v>435</v>
+      </c>
+      <c r="B12" s="5">
+        <v>1</v>
+      </c>
+      <c r="C12" s="2" t="s">
         <v>389</v>
       </c>
-      <c r="D12" s="1" t="s">
-        <v>4</v>
+      <c r="D12" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>436</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
-        <v>437</v>
+        <v>405</v>
       </c>
       <c r="B13" s="5">
         <v>1</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>389</v>
+        <v>407</v>
       </c>
       <c r="D13" s="5" t="s">
         <v>4</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>438</v>
+        <v>406</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
-        <v>406</v>
+        <v>415</v>
       </c>
       <c r="B14" s="5">
         <v>1</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="D14" s="5" t="s">
         <v>4</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>407</v>
+        <v>416</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
-        <v>416</v>
+        <v>25</v>
       </c>
       <c r="B15" s="5">
         <v>1</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>408</v>
+        <v>11</v>
       </c>
       <c r="D15" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="E15" s="5" t="s">
-        <v>417</v>
-      </c>
+      <c r="E15" s="5"/>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A16" s="8" t="s">
-        <v>25</v>
-      </c>
-      <c r="C16" t="s">
+      <c r="A16" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B16" s="5">
+        <v>1</v>
+      </c>
+      <c r="C16" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="D16" s="1" t="s">
-        <v>4</v>
+      <c r="D16" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="E16" s="5" t="s">
+        <v>538</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A17" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="C17" t="s">
+      <c r="A17" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B17" s="5">
+        <v>1</v>
+      </c>
+      <c r="C17" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="D17" s="1" t="s">
-        <v>4</v>
+      <c r="D17" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="E17" s="5" t="s">
+        <v>198</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A18" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="C18" t="s">
+      <c r="A18" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B18" s="5">
+        <v>1</v>
+      </c>
+      <c r="C18" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="D18" s="1" t="s">
-        <v>4</v>
+      <c r="D18" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="E18" s="5" t="s">
+        <v>539</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A19" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="C19" t="s">
+      <c r="A19" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="B19" s="5">
+        <v>1</v>
+      </c>
+      <c r="C19" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="D19" s="1" t="s">
-        <v>4</v>
+      <c r="D19" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="E19" s="5" t="s">
+        <v>132</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
-        <v>131</v>
+        <v>362</v>
       </c>
       <c r="B20" s="5">
         <v>1</v>
@@ -5901,12 +5940,12 @@
         <v>4</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>132</v>
+        <v>363</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="B21" s="5">
         <v>1</v>
@@ -5918,12 +5957,12 @@
         <v>4</v>
       </c>
       <c r="E21" s="5" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="B22" s="5">
         <v>1</v>
@@ -5935,12 +5974,12 @@
         <v>4</v>
       </c>
       <c r="E22" s="5" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="B23" s="5">
         <v>1</v>
@@ -5952,12 +5991,12 @@
         <v>4</v>
       </c>
       <c r="E23" s="5" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="B24" s="5">
         <v>1</v>
@@ -5969,12 +6008,12 @@
         <v>4</v>
       </c>
       <c r="E24" s="5" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="B25" s="5">
         <v>1</v>
@@ -5986,12 +6025,12 @@
         <v>4</v>
       </c>
       <c r="E25" s="5" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="3" t="s">
-        <v>372</v>
+        <v>376</v>
       </c>
       <c r="B26" s="5">
         <v>1</v>
@@ -6003,12 +6042,12 @@
         <v>4</v>
       </c>
       <c r="E26" s="5" t="s">
-        <v>373</v>
+        <v>377</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="B27" s="5">
         <v>1</v>
@@ -6020,12 +6059,12 @@
         <v>4</v>
       </c>
       <c r="E27" s="5" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="3" t="s">
-        <v>378</v>
+        <v>382</v>
       </c>
       <c r="B28" s="5">
         <v>1</v>
@@ -6037,51 +6076,61 @@
         <v>4</v>
       </c>
       <c r="E28" s="5" t="s">
-        <v>379</v>
+        <v>383</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
-        <v>382</v>
+        <v>20</v>
       </c>
       <c r="B29" s="5">
         <v>1</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="D29" s="5" t="s">
         <v>4</v>
       </c>
       <c r="E29" s="5" t="s">
-        <v>383</v>
+        <v>541</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A30" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="C30" t="s">
+      <c r="A30" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B30" s="5">
+        <v>1</v>
+      </c>
+      <c r="C30" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="D30" s="1" t="s">
-        <v>4</v>
-      </c>
+      <c r="D30" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="E30" s="5"/>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A31" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="C31" t="s">
+      <c r="A31" s="3" t="s">
+        <v>352</v>
+      </c>
+      <c r="B31" s="5">
+        <v>1</v>
+      </c>
+      <c r="C31" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="D31" s="1" t="s">
-        <v>4</v>
+      <c r="D31" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="E31" s="5" t="s">
+        <v>353</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" s="3" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="B32" s="5">
         <v>1</v>
@@ -6093,12 +6142,12 @@
         <v>4</v>
       </c>
       <c r="E32" s="5" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="3" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="B33" s="5">
         <v>1</v>
@@ -6110,12 +6159,12 @@
         <v>4</v>
       </c>
       <c r="E33" s="5" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" s="3" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="B34" s="5">
         <v>1</v>
@@ -6127,12 +6176,12 @@
         <v>4</v>
       </c>
       <c r="E34" s="5" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" s="3" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="B35" s="5">
         <v>1</v>
@@ -6144,12 +6193,12 @@
         <v>4</v>
       </c>
       <c r="E35" s="5" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" s="3" t="s">
-        <v>360</v>
+        <v>417</v>
       </c>
       <c r="B36" s="5">
         <v>1</v>
@@ -6161,7 +6210,7 @@
         <v>4</v>
       </c>
       <c r="E36" s="5" t="s">
-        <v>361</v>
+        <v>418</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
@@ -6183,7 +6232,7 @@
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" s="3" t="s">
-        <v>421</v>
+        <v>433</v>
       </c>
       <c r="B38" s="5">
         <v>1</v>
@@ -6194,36 +6243,38 @@
       <c r="D38" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="E38" s="5" t="s">
-        <v>422</v>
-      </c>
+      <c r="E38" s="5"/>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A39" s="8" t="s">
-        <v>435</v>
-      </c>
-      <c r="B39" s="1">
-        <v>1</v>
-      </c>
-      <c r="C39" t="s">
+      <c r="A39" s="3" t="s">
+        <v>434</v>
+      </c>
+      <c r="B39" s="5">
+        <v>1</v>
+      </c>
+      <c r="C39" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="D39" s="1" t="s">
-        <v>4</v>
-      </c>
+      <c r="D39" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="E39" s="5"/>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A40" s="8" t="s">
-        <v>436</v>
-      </c>
-      <c r="B40" s="1">
-        <v>1</v>
-      </c>
-      <c r="C40" t="s">
+      <c r="A40" s="3" t="s">
+        <v>446</v>
+      </c>
+      <c r="B40" s="5">
+        <v>1</v>
+      </c>
+      <c r="C40" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="D40" s="1" t="s">
-        <v>4</v>
+      <c r="D40" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="E40" s="5" t="s">
+        <v>447</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
@@ -6240,35 +6291,35 @@
         <v>4</v>
       </c>
       <c r="E41" s="5" t="s">
-        <v>449</v>
+        <v>285</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" s="3" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="B42" s="5">
         <v>1</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>21</v>
+        <v>452</v>
       </c>
       <c r="D42" s="5" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E42" s="5" t="s">
-        <v>285</v>
+        <v>453</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" s="3" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="B43" s="5">
         <v>1</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>454</v>
+        <v>452</v>
       </c>
       <c r="D43" s="5" t="s">
         <v>2</v>
@@ -6279,38 +6330,39 @@
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" s="3" t="s">
-        <v>456</v>
+        <v>460</v>
       </c>
       <c r="B44" s="5">
         <v>1</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>454</v>
+        <v>452</v>
       </c>
       <c r="D44" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="E44" s="5" t="s">
-        <v>457</v>
-      </c>
+      <c r="E44" s="5"/>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A45" s="8" t="s">
-        <v>462</v>
-      </c>
-      <c r="B45" s="1">
-        <v>1</v>
-      </c>
-      <c r="C45" t="s">
-        <v>454</v>
-      </c>
-      <c r="D45" s="1" t="s">
-        <v>2</v>
+      <c r="A45" s="3" t="s">
+        <v>390</v>
+      </c>
+      <c r="B45" s="5">
+        <v>1</v>
+      </c>
+      <c r="C45" s="2" t="s">
+        <v>389</v>
+      </c>
+      <c r="D45" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="E45" s="5" t="s">
+        <v>391</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" s="3" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="B46" s="5">
         <v>1</v>
@@ -6321,194 +6373,231 @@
       <c r="D46" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="E46" s="5" t="s">
-        <v>391</v>
-      </c>
+      <c r="E46" s="5"/>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A47" s="8" t="s">
-        <v>392</v>
-      </c>
-      <c r="B47" s="1">
-        <v>1</v>
-      </c>
-      <c r="C47" t="s">
+      <c r="A47" s="3" t="s">
+        <v>394</v>
+      </c>
+      <c r="B47" s="5">
+        <v>1</v>
+      </c>
+      <c r="C47" s="2" t="s">
         <v>389</v>
       </c>
-      <c r="D47" s="1" t="s">
-        <v>2</v>
-      </c>
+      <c r="D47" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="E47" s="5"/>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A48" s="8" t="s">
+      <c r="A48" s="3" t="s">
         <v>395</v>
       </c>
-      <c r="B48" s="1">
-        <v>1</v>
-      </c>
-      <c r="C48" t="s">
+      <c r="B48" s="5">
+        <v>1</v>
+      </c>
+      <c r="C48" s="2" t="s">
         <v>389</v>
       </c>
-      <c r="D48" s="1" t="s">
-        <v>2</v>
+      <c r="D48" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="E48" s="5" t="s">
+        <v>396</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" s="3" t="s">
-        <v>396</v>
+        <v>410</v>
       </c>
       <c r="B49" s="5">
         <v>1</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>389</v>
+        <v>407</v>
       </c>
       <c r="D49" s="5" t="s">
         <v>2</v>
       </c>
       <c r="E49" s="5" t="s">
-        <v>397</v>
+        <v>411</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" s="3" t="s">
-        <v>411</v>
+        <v>414</v>
       </c>
       <c r="B50" s="5">
         <v>1</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="D50" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="E50" s="5" t="s">
-        <v>412</v>
-      </c>
+      <c r="E50" s="5"/>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A51" s="8" t="s">
-        <v>415</v>
-      </c>
-      <c r="B51" s="1">
-        <v>1</v>
-      </c>
-      <c r="C51" t="s">
-        <v>408</v>
-      </c>
-      <c r="D51" s="1" t="s">
-        <v>2</v>
+      <c r="A51" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B51" s="5">
+        <v>1</v>
+      </c>
+      <c r="C51" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D51" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="E51" s="5" t="s">
+        <v>198</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A52" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="C52" t="s">
+      <c r="A52" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B52" s="5">
+        <v>1</v>
+      </c>
+      <c r="C52" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="D52" s="1" t="s">
-        <v>2</v>
-      </c>
+      <c r="D52" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="E52" s="5"/>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A53" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="C53" t="s">
+      <c r="A53" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B53" s="5">
+        <v>1</v>
+      </c>
+      <c r="C53" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="D53" s="1" t="s">
-        <v>2</v>
-      </c>
+      <c r="D53" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="E53" s="5"/>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A54" s="8" t="s">
-        <v>27</v>
-      </c>
-      <c r="C54" t="s">
+      <c r="A54" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B54" s="5">
+        <v>1</v>
+      </c>
+      <c r="C54" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="D54" s="1" t="s">
-        <v>2</v>
-      </c>
+      <c r="D54" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="E54" s="5"/>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A55" s="8" t="s">
-        <v>26</v>
-      </c>
-      <c r="C55" t="s">
+      <c r="A55" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B55" s="5">
+        <v>1</v>
+      </c>
+      <c r="C55" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="D55" s="1" t="s">
-        <v>2</v>
-      </c>
+      <c r="D55" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="E55" s="5"/>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A56" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="C56" t="s">
+      <c r="A56" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B56" s="5">
+        <v>1</v>
+      </c>
+      <c r="C56" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="D56" s="1" t="s">
-        <v>2</v>
-      </c>
+      <c r="D56" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="E56" s="5"/>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A57" s="8" t="s">
-        <v>30</v>
-      </c>
-      <c r="C57" t="s">
+      <c r="A57" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="B57" s="5">
+        <v>1</v>
+      </c>
+      <c r="C57" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="D57" s="1" t="s">
-        <v>2</v>
-      </c>
+      <c r="D57" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="E57" s="5"/>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A58" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="C58" t="s">
+      <c r="A58" s="3" t="s">
+        <v>374</v>
+      </c>
+      <c r="B58" s="5">
+        <v>1</v>
+      </c>
+      <c r="C58" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="D58" s="1" t="s">
-        <v>2</v>
-      </c>
+      <c r="D58" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="E58" s="5"/>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A59" s="8" t="s">
-        <v>374</v>
-      </c>
-      <c r="B59" s="1">
-        <v>1</v>
-      </c>
-      <c r="C59" t="s">
+      <c r="A59" s="3" t="s">
+        <v>375</v>
+      </c>
+      <c r="B59" s="5">
+        <v>1</v>
+      </c>
+      <c r="C59" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="D59" s="1" t="s">
-        <v>2</v>
+      <c r="D59" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="E59" s="5" t="s">
+        <v>540</v>
       </c>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A60" s="8" t="s">
-        <v>375</v>
-      </c>
-      <c r="B60" s="1">
-        <v>1</v>
-      </c>
-      <c r="C60" t="s">
+      <c r="A60" s="3" t="s">
+        <v>380</v>
+      </c>
+      <c r="B60" s="5">
+        <v>1</v>
+      </c>
+      <c r="C60" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="D60" s="1" t="s">
-        <v>2</v>
+      <c r="D60" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="E60" s="5" t="s">
+        <v>381</v>
       </c>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A61" s="3" t="s">
-        <v>380</v>
+        <v>384</v>
       </c>
       <c r="B61" s="5">
         <v>1</v>
@@ -6520,12 +6609,12 @@
         <v>2</v>
       </c>
       <c r="E61" s="5" t="s">
-        <v>381</v>
+        <v>385</v>
       </c>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A62" s="3" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="B62" s="5">
         <v>1</v>
@@ -6537,12 +6626,12 @@
         <v>2</v>
       </c>
       <c r="E62" s="5" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A63" s="3" t="s">
-        <v>386</v>
+        <v>428</v>
       </c>
       <c r="B63" s="5">
         <v>1</v>
@@ -6553,29 +6642,32 @@
       <c r="D63" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="E63" s="5" t="s">
-        <v>387</v>
-      </c>
+      <c r="E63" s="5"/>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A64" s="8" t="s">
-        <v>430</v>
-      </c>
-      <c r="B64" s="1">
-        <v>1</v>
-      </c>
-      <c r="C64" t="s">
-        <v>11</v>
-      </c>
-      <c r="D64" s="1" t="s">
-        <v>2</v>
+      <c r="A64" s="3" t="s">
+        <v>349</v>
+      </c>
+      <c r="B64" s="5">
+        <v>1</v>
+      </c>
+      <c r="C64" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D64" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="E64" s="5" t="s">
+        <v>350</v>
       </c>
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A65" s="3" t="s">
         <v>349</v>
       </c>
-      <c r="B65" s="5"/>
+      <c r="B65" s="5">
+        <v>1</v>
+      </c>
       <c r="C65" s="2" t="s">
         <v>21</v>
       </c>
@@ -6583,14 +6675,16 @@
         <v>2</v>
       </c>
       <c r="E65" s="5" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A66" s="3" t="s">
-        <v>349</v>
-      </c>
-      <c r="B66" s="5"/>
+        <v>421</v>
+      </c>
+      <c r="B66" s="5">
+        <v>1</v>
+      </c>
       <c r="C66" s="2" t="s">
         <v>21</v>
       </c>
@@ -6598,7 +6692,7 @@
         <v>2</v>
       </c>
       <c r="E66" s="5" t="s">
-        <v>351</v>
+        <v>422</v>
       </c>
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.25">
@@ -6608,13 +6702,13 @@
       <c r="B67" s="5">
         <v>1</v>
       </c>
-      <c r="C67" s="2" t="s">
+      <c r="C67" s="4" t="s">
         <v>21</v>
       </c>
       <c r="D67" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="E67" s="5" t="s">
+      <c r="E67" s="7" t="s">
         <v>424</v>
       </c>
     </row>
@@ -6625,13 +6719,13 @@
       <c r="B68" s="5">
         <v>1</v>
       </c>
-      <c r="C68" s="4" t="s">
+      <c r="C68" s="2" t="s">
         <v>21</v>
       </c>
       <c r="D68" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="E68" s="7" t="s">
+      <c r="E68" s="5" t="s">
         <v>426</v>
       </c>
     </row>
@@ -6648,27 +6742,28 @@
       <c r="D69" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="E69" s="5" t="s">
-        <v>428</v>
-      </c>
+      <c r="E69" s="5"/>
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A70" s="8" t="s">
+      <c r="A70" s="3" t="s">
         <v>429</v>
       </c>
-      <c r="B70" s="1">
-        <v>1</v>
-      </c>
-      <c r="C70" t="s">
+      <c r="B70" s="5">
+        <v>1</v>
+      </c>
+      <c r="C70" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="D70" s="1" t="s">
-        <v>2</v>
+      <c r="D70" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="E70" s="5" t="s">
+        <v>430</v>
       </c>
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A71" s="3" t="s">
-        <v>431</v>
+        <v>437</v>
       </c>
       <c r="B71" s="5">
         <v>1</v>
@@ -6680,7 +6775,7 @@
         <v>2</v>
       </c>
       <c r="E71" s="5" t="s">
-        <v>432</v>
+        <v>438</v>
       </c>
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.25">
@@ -6697,12 +6792,12 @@
         <v>2</v>
       </c>
       <c r="E72" s="5" t="s">
-        <v>440</v>
+        <v>409</v>
       </c>
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A73" s="3" t="s">
-        <v>441</v>
+        <v>444</v>
       </c>
       <c r="B73" s="5">
         <v>1</v>
@@ -6714,12 +6809,12 @@
         <v>2</v>
       </c>
       <c r="E73" s="5" t="s">
-        <v>410</v>
+        <v>285</v>
       </c>
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A74" s="3" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="B74" s="5">
         <v>1</v>
@@ -6730,156 +6825,124 @@
       <c r="D74" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="E74" s="5" t="s">
-        <v>285</v>
-      </c>
+      <c r="E74" s="5"/>
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A75" s="8" t="s">
-        <v>447</v>
-      </c>
-      <c r="B75" s="1">
-        <v>1</v>
-      </c>
-      <c r="C75" t="s">
+      <c r="A75" s="3" t="s">
+        <v>449</v>
+      </c>
+      <c r="B75" s="5">
+        <v>1</v>
+      </c>
+      <c r="C75" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="D75" s="1" t="s">
-        <v>2</v>
+      <c r="D75" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="E75" s="5" t="s">
+        <v>450</v>
       </c>
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A76" s="3" t="s">
-        <v>451</v>
+        <v>408</v>
       </c>
       <c r="B76" s="5">
         <v>1</v>
       </c>
       <c r="C76" s="2" t="s">
-        <v>21</v>
+        <v>407</v>
       </c>
       <c r="D76" s="5" t="s">
         <v>2</v>
       </c>
       <c r="E76" s="5" t="s">
-        <v>452</v>
-      </c>
-    </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A77" s="8" t="s">
-        <v>418</v>
-      </c>
-      <c r="B77" s="1">
-        <v>1</v>
-      </c>
-      <c r="C77" t="s">
-        <v>216</v>
-      </c>
-      <c r="D77" s="1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A78" s="3" t="s">
         <v>409</v>
-      </c>
-      <c r="B78" s="5">
-        <v>1</v>
-      </c>
-      <c r="C78" s="2" t="s">
-        <v>408</v>
-      </c>
-      <c r="D78" s="5" t="s">
-        <v>2</v>
-      </c>
-      <c r="E78" s="5" t="s">
-        <v>410</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A20" r:id="rId1" xr:uid="{21D25134-52B4-4BAA-B487-A621F9BC4E41}"/>
-    <hyperlink ref="A22" r:id="rId2" xr:uid="{C75924C8-212C-4126-8C51-474FEA0052FD}"/>
+    <hyperlink ref="A19" r:id="rId1" xr:uid="{21D25134-52B4-4BAA-B487-A621F9BC4E41}"/>
+    <hyperlink ref="A21" r:id="rId2" xr:uid="{C75924C8-212C-4126-8C51-474FEA0052FD}"/>
     <hyperlink ref="A11" r:id="rId3" xr:uid="{87C6A6CF-564B-42A4-8248-3FCF86107E16}"/>
-    <hyperlink ref="A49" r:id="rId4" xr:uid="{5A87060B-63DF-4E27-B8EB-A3030884F759}"/>
-    <hyperlink ref="A78" r:id="rId5" xr:uid="{07920AE6-F744-4463-AB3F-EFB9F5EBE685}"/>
-    <hyperlink ref="A77" r:id="rId6" xr:uid="{DB8137EB-81CD-4DC2-8C7C-2B5C4EE0D41E}"/>
-    <hyperlink ref="A76" r:id="rId7" xr:uid="{F7C05217-5A82-458F-BA27-01E40C5EF9C0}"/>
-    <hyperlink ref="A75" r:id="rId8" xr:uid="{97D435C8-50CB-4854-8683-7E771B63DBF4}"/>
-    <hyperlink ref="A74" r:id="rId9" xr:uid="{B5706F29-02B5-4BA1-99C0-A9B51D97DF9F}"/>
-    <hyperlink ref="A73" r:id="rId10" xr:uid="{FEA625D5-5987-479C-BCF8-705E37DA58CC}"/>
-    <hyperlink ref="A72" r:id="rId11" xr:uid="{4E9CF9AC-DD7A-44C2-BDFB-E51E6A349D3C}"/>
-    <hyperlink ref="A71" r:id="rId12" xr:uid="{155D1C6E-579E-4E25-9F85-884ED5956C41}"/>
-    <hyperlink ref="A70" r:id="rId13" xr:uid="{F2EBAF24-F0DE-4F30-8155-7495CEEA44C7}"/>
-    <hyperlink ref="A69" r:id="rId14" xr:uid="{EC74BD60-8496-4246-8750-64391EB365BB}"/>
-    <hyperlink ref="A68" r:id="rId15" xr:uid="{1020E8CE-A83B-4CE1-8ECF-F52D77A795AE}"/>
-    <hyperlink ref="A67" r:id="rId16" xr:uid="{BC228CCF-F637-4B39-A5EF-7F3E7A44CCDE}"/>
-    <hyperlink ref="A66" r:id="rId17" xr:uid="{88591B95-93B5-496D-A4B8-320E4B349F45}"/>
-    <hyperlink ref="A65" r:id="rId18" xr:uid="{2900AD04-38BF-4418-BBC6-F4333DFEB25B}"/>
-    <hyperlink ref="A64" r:id="rId19" xr:uid="{A33A354F-4660-4552-96C3-ECF2DAC54F77}"/>
-    <hyperlink ref="A63" r:id="rId20" xr:uid="{C857C978-C6E6-42BE-9F40-B153AB84B17F}"/>
-    <hyperlink ref="A62" r:id="rId21" xr:uid="{7DCFC8EB-D8C5-46EC-99F9-A53E52C8B707}"/>
-    <hyperlink ref="A61" r:id="rId22" xr:uid="{68578F20-7BEC-4BEA-8804-B5C2AA4CC1EB}"/>
-    <hyperlink ref="A60" r:id="rId23" xr:uid="{2EAD7991-115A-4492-9D71-6F88F7DFD03A}"/>
-    <hyperlink ref="A59" r:id="rId24" xr:uid="{39C0DD33-FCAC-4CC6-A788-CEBAFA72D162}"/>
-    <hyperlink ref="A58" r:id="rId25" xr:uid="{5074072E-4829-4F04-86E4-FF838A2DB1C1}"/>
-    <hyperlink ref="A57" r:id="rId26" xr:uid="{439975E3-37D1-4A45-887A-B83E463B7C55}"/>
-    <hyperlink ref="A56" r:id="rId27" xr:uid="{53C0BA17-8195-47A8-A9DA-2EB5C6119F0D}"/>
-    <hyperlink ref="A55" r:id="rId28" xr:uid="{BC70362B-DC21-469C-AAA0-7D54B6066211}"/>
-    <hyperlink ref="A54" r:id="rId29" xr:uid="{09A7C60F-C9B8-490A-AF17-B9522D30D0FC}"/>
-    <hyperlink ref="A53" r:id="rId30" xr:uid="{673AFC5F-1893-431F-B672-7F082257E253}"/>
-    <hyperlink ref="A52" r:id="rId31" xr:uid="{BDB388B9-D5EC-419A-A7D0-64F2AE2E580A}"/>
-    <hyperlink ref="A51" r:id="rId32" xr:uid="{B57ACB21-1DB4-4F38-AF58-D34776E965F3}"/>
-    <hyperlink ref="A50" r:id="rId33" xr:uid="{FFC376C9-3B07-456D-9B5D-C46926FB1F89}"/>
-    <hyperlink ref="A48" r:id="rId34" xr:uid="{D246E8E5-3A6A-44B5-AAD2-44024A07E36F}"/>
-    <hyperlink ref="A47" r:id="rId35" xr:uid="{B765E4A0-B8A5-412F-ABDC-B2E360C2AFBB}"/>
-    <hyperlink ref="A46" r:id="rId36" xr:uid="{941774A7-7BB2-4BF4-BDF5-87AE80343D8C}"/>
-    <hyperlink ref="A45" r:id="rId37" xr:uid="{3A2DA735-DFD9-44C8-87D0-297858B2116B}"/>
-    <hyperlink ref="A44" r:id="rId38" xr:uid="{B3ED65ED-C243-4683-BD26-C897A6D0D348}"/>
-    <hyperlink ref="A43" r:id="rId39" xr:uid="{452905BB-4E4C-46AD-8C02-1FC1B0C058EE}"/>
-    <hyperlink ref="A42" r:id="rId40" xr:uid="{EDED8E91-8EAB-4AE4-BB03-016D6F13BD4E}"/>
-    <hyperlink ref="A41" r:id="rId41" xr:uid="{B7E10220-607F-4E84-A4DB-DDA70F0EED4C}"/>
-    <hyperlink ref="A40" r:id="rId42" xr:uid="{6BA74B94-3C28-49B0-BC5E-53B57CB87DB2}"/>
-    <hyperlink ref="A39" r:id="rId43" xr:uid="{24828B66-EC91-4A40-9FE3-FE24077C4A72}"/>
-    <hyperlink ref="A38" r:id="rId44" xr:uid="{E5D4BB8C-D3EA-4F8D-974F-A7C8C2F2ACF0}"/>
-    <hyperlink ref="A37" r:id="rId45" xr:uid="{50F42924-666E-4039-9CB3-D435E8DE2C44}"/>
-    <hyperlink ref="A36" r:id="rId46" xr:uid="{20CA3FE3-CF25-4B1E-9044-05E71D6BBCC8}"/>
-    <hyperlink ref="A35" r:id="rId47" xr:uid="{1BCB6CDD-7AF2-4EF7-BEFE-6ED650A63067}"/>
-    <hyperlink ref="A34" r:id="rId48" xr:uid="{5D23EEF9-4FD3-4D00-9AB0-1C00C454F057}"/>
-    <hyperlink ref="A33" r:id="rId49" xr:uid="{45FC349D-E5AA-43F5-BC41-3CB69A5CFC3B}"/>
-    <hyperlink ref="A32" r:id="rId50" xr:uid="{F460B329-1B4E-4C6E-94AF-57305CB84736}"/>
-    <hyperlink ref="A31" r:id="rId51" xr:uid="{C8B7B629-692D-4DBC-9201-296CAA6749A1}"/>
-    <hyperlink ref="A30" r:id="rId52" xr:uid="{0B723F85-47CF-4A63-AC75-AAD32280D756}"/>
-    <hyperlink ref="A29" r:id="rId53" xr:uid="{DEF7D370-D59D-4A30-BE30-53E5D234D01F}"/>
-    <hyperlink ref="A28" r:id="rId54" xr:uid="{B053EC5F-A596-4CBB-B2C6-533D05FDFFEB}"/>
-    <hyperlink ref="A27" r:id="rId55" xr:uid="{B1AC30D2-D9D6-4E68-BAE1-A937B933D6B4}"/>
-    <hyperlink ref="A26" r:id="rId56" xr:uid="{04E91419-240C-4C40-9CE4-51B5DE4C320C}"/>
-    <hyperlink ref="A25" r:id="rId57" xr:uid="{224F3FDA-6133-438C-9645-6543A32D404A}"/>
-    <hyperlink ref="A24" r:id="rId58" xr:uid="{A4F61A63-0C4F-4E23-BFAE-E9CC69935EF2}"/>
-    <hyperlink ref="A23" r:id="rId59" xr:uid="{EA1DCE00-6252-4B38-B38B-CC6F401BD05B}"/>
-    <hyperlink ref="A21" r:id="rId60" xr:uid="{74330122-414A-4EE6-B7D1-633978CAFC7F}"/>
-    <hyperlink ref="A19" r:id="rId61" xr:uid="{646431EC-C544-4C5B-9C8B-33FA5C080A5B}"/>
-    <hyperlink ref="A18" r:id="rId62" xr:uid="{7AED7DC4-C836-4A03-A289-3731E38BA141}"/>
-    <hyperlink ref="A17" r:id="rId63" xr:uid="{F02129EB-2BBD-443E-9D69-6623A732C49F}"/>
-    <hyperlink ref="A16" r:id="rId64" xr:uid="{424CD5D2-5B3D-46A5-8723-D7AEB663A399}"/>
-    <hyperlink ref="A15" r:id="rId65" xr:uid="{55EF3F12-9C12-468F-B2F7-48B4187B239A}"/>
-    <hyperlink ref="A14" r:id="rId66" xr:uid="{DC84D70E-A9B3-4945-AF4F-0D220AD052C1}"/>
-    <hyperlink ref="A13" r:id="rId67" xr:uid="{680F938F-34DD-4AB6-99C0-A237DBA25C40}"/>
-    <hyperlink ref="A12" r:id="rId68" xr:uid="{2D6F6571-524D-49DF-A753-79BBF49FFC3E}"/>
-    <hyperlink ref="A10" r:id="rId69" xr:uid="{F3B2B3FC-3652-463F-AC4B-24093389FED6}"/>
-    <hyperlink ref="A9" r:id="rId70" xr:uid="{52FFDFB6-8BA7-440C-AB0A-C2CC4D263F1D}"/>
-    <hyperlink ref="A8" r:id="rId71" xr:uid="{0B717454-34EB-457E-81FA-5F083E19D92F}"/>
-    <hyperlink ref="A7" r:id="rId72" xr:uid="{79193D90-FBAC-42CF-884B-1B287D33D289}"/>
-    <hyperlink ref="A6" r:id="rId73" xr:uid="{D2388750-EFD9-405D-86AE-BCE3CA89E04B}"/>
-    <hyperlink ref="A5" r:id="rId74" xr:uid="{BAED895C-B388-419D-AA42-EAC5180A469B}"/>
-    <hyperlink ref="A4" r:id="rId75" xr:uid="{444CE840-7C67-4021-86DD-17B2E2040CE2}"/>
-    <hyperlink ref="A3" r:id="rId76" xr:uid="{C46F5ED2-A800-437B-9907-79AB5BC3088C}"/>
-    <hyperlink ref="A2" r:id="rId77" xr:uid="{6A0E4EEF-6185-474B-8E18-1E72C0181781}"/>
+    <hyperlink ref="A48" r:id="rId4" xr:uid="{5A87060B-63DF-4E27-B8EB-A3030884F759}"/>
+    <hyperlink ref="A76" r:id="rId5" xr:uid="{07920AE6-F744-4463-AB3F-EFB9F5EBE685}"/>
+    <hyperlink ref="A75" r:id="rId6" xr:uid="{F7C05217-5A82-458F-BA27-01E40C5EF9C0}"/>
+    <hyperlink ref="A74" r:id="rId7" xr:uid="{97D435C8-50CB-4854-8683-7E771B63DBF4}"/>
+    <hyperlink ref="A73" r:id="rId8" xr:uid="{B5706F29-02B5-4BA1-99C0-A9B51D97DF9F}"/>
+    <hyperlink ref="A72" r:id="rId9" xr:uid="{FEA625D5-5987-479C-BCF8-705E37DA58CC}"/>
+    <hyperlink ref="A71" r:id="rId10" xr:uid="{4E9CF9AC-DD7A-44C2-BDFB-E51E6A349D3C}"/>
+    <hyperlink ref="A70" r:id="rId11" xr:uid="{155D1C6E-579E-4E25-9F85-884ED5956C41}"/>
+    <hyperlink ref="A69" r:id="rId12" xr:uid="{F2EBAF24-F0DE-4F30-8155-7495CEEA44C7}"/>
+    <hyperlink ref="A68" r:id="rId13" xr:uid="{EC74BD60-8496-4246-8750-64391EB365BB}"/>
+    <hyperlink ref="A67" r:id="rId14" xr:uid="{1020E8CE-A83B-4CE1-8ECF-F52D77A795AE}"/>
+    <hyperlink ref="A66" r:id="rId15" xr:uid="{BC228CCF-F637-4B39-A5EF-7F3E7A44CCDE}"/>
+    <hyperlink ref="A65" r:id="rId16" xr:uid="{88591B95-93B5-496D-A4B8-320E4B349F45}"/>
+    <hyperlink ref="A64" r:id="rId17" xr:uid="{2900AD04-38BF-4418-BBC6-F4333DFEB25B}"/>
+    <hyperlink ref="A63" r:id="rId18" xr:uid="{A33A354F-4660-4552-96C3-ECF2DAC54F77}"/>
+    <hyperlink ref="A62" r:id="rId19" xr:uid="{C857C978-C6E6-42BE-9F40-B153AB84B17F}"/>
+    <hyperlink ref="A61" r:id="rId20" xr:uid="{7DCFC8EB-D8C5-46EC-99F9-A53E52C8B707}"/>
+    <hyperlink ref="A60" r:id="rId21" xr:uid="{68578F20-7BEC-4BEA-8804-B5C2AA4CC1EB}"/>
+    <hyperlink ref="A59" r:id="rId22" xr:uid="{2EAD7991-115A-4492-9D71-6F88F7DFD03A}"/>
+    <hyperlink ref="A58" r:id="rId23" xr:uid="{39C0DD33-FCAC-4CC6-A788-CEBAFA72D162}"/>
+    <hyperlink ref="A57" r:id="rId24" xr:uid="{5074072E-4829-4F04-86E4-FF838A2DB1C1}"/>
+    <hyperlink ref="A56" r:id="rId25" xr:uid="{439975E3-37D1-4A45-887A-B83E463B7C55}"/>
+    <hyperlink ref="A55" r:id="rId26" xr:uid="{53C0BA17-8195-47A8-A9DA-2EB5C6119F0D}"/>
+    <hyperlink ref="A54" r:id="rId27" xr:uid="{BC70362B-DC21-469C-AAA0-7D54B6066211}"/>
+    <hyperlink ref="A53" r:id="rId28" xr:uid="{09A7C60F-C9B8-490A-AF17-B9522D30D0FC}"/>
+    <hyperlink ref="A52" r:id="rId29" xr:uid="{673AFC5F-1893-431F-B672-7F082257E253}"/>
+    <hyperlink ref="A51" r:id="rId30" xr:uid="{BDB388B9-D5EC-419A-A7D0-64F2AE2E580A}"/>
+    <hyperlink ref="A50" r:id="rId31" xr:uid="{B57ACB21-1DB4-4F38-AF58-D34776E965F3}"/>
+    <hyperlink ref="A49" r:id="rId32" xr:uid="{FFC376C9-3B07-456D-9B5D-C46926FB1F89}"/>
+    <hyperlink ref="A47" r:id="rId33" xr:uid="{D246E8E5-3A6A-44B5-AAD2-44024A07E36F}"/>
+    <hyperlink ref="A46" r:id="rId34" xr:uid="{B765E4A0-B8A5-412F-ABDC-B2E360C2AFBB}"/>
+    <hyperlink ref="A45" r:id="rId35" xr:uid="{941774A7-7BB2-4BF4-BDF5-87AE80343D8C}"/>
+    <hyperlink ref="A44" r:id="rId36" xr:uid="{3A2DA735-DFD9-44C8-87D0-297858B2116B}"/>
+    <hyperlink ref="A43" r:id="rId37" xr:uid="{B3ED65ED-C243-4683-BD26-C897A6D0D348}"/>
+    <hyperlink ref="A42" r:id="rId38" xr:uid="{452905BB-4E4C-46AD-8C02-1FC1B0C058EE}"/>
+    <hyperlink ref="A41" r:id="rId39" xr:uid="{EDED8E91-8EAB-4AE4-BB03-016D6F13BD4E}"/>
+    <hyperlink ref="A40" r:id="rId40" xr:uid="{B7E10220-607F-4E84-A4DB-DDA70F0EED4C}"/>
+    <hyperlink ref="A39" r:id="rId41" xr:uid="{6BA74B94-3C28-49B0-BC5E-53B57CB87DB2}"/>
+    <hyperlink ref="A38" r:id="rId42" xr:uid="{24828B66-EC91-4A40-9FE3-FE24077C4A72}"/>
+    <hyperlink ref="A37" r:id="rId43" xr:uid="{E5D4BB8C-D3EA-4F8D-974F-A7C8C2F2ACF0}"/>
+    <hyperlink ref="A36" r:id="rId44" xr:uid="{50F42924-666E-4039-9CB3-D435E8DE2C44}"/>
+    <hyperlink ref="A35" r:id="rId45" xr:uid="{20CA3FE3-CF25-4B1E-9044-05E71D6BBCC8}"/>
+    <hyperlink ref="A34" r:id="rId46" xr:uid="{1BCB6CDD-7AF2-4EF7-BEFE-6ED650A63067}"/>
+    <hyperlink ref="A33" r:id="rId47" xr:uid="{5D23EEF9-4FD3-4D00-9AB0-1C00C454F057}"/>
+    <hyperlink ref="A32" r:id="rId48" xr:uid="{45FC349D-E5AA-43F5-BC41-3CB69A5CFC3B}"/>
+    <hyperlink ref="A31" r:id="rId49" xr:uid="{F460B329-1B4E-4C6E-94AF-57305CB84736}"/>
+    <hyperlink ref="A30" r:id="rId50" xr:uid="{C8B7B629-692D-4DBC-9201-296CAA6749A1}"/>
+    <hyperlink ref="A29" r:id="rId51" xr:uid="{0B723F85-47CF-4A63-AC75-AAD32280D756}"/>
+    <hyperlink ref="A28" r:id="rId52" xr:uid="{DEF7D370-D59D-4A30-BE30-53E5D234D01F}"/>
+    <hyperlink ref="A27" r:id="rId53" xr:uid="{B053EC5F-A596-4CBB-B2C6-533D05FDFFEB}"/>
+    <hyperlink ref="A26" r:id="rId54" xr:uid="{B1AC30D2-D9D6-4E68-BAE1-A937B933D6B4}"/>
+    <hyperlink ref="A25" r:id="rId55" xr:uid="{04E91419-240C-4C40-9CE4-51B5DE4C320C}"/>
+    <hyperlink ref="A24" r:id="rId56" xr:uid="{224F3FDA-6133-438C-9645-6543A32D404A}"/>
+    <hyperlink ref="A23" r:id="rId57" xr:uid="{A4F61A63-0C4F-4E23-BFAE-E9CC69935EF2}"/>
+    <hyperlink ref="A22" r:id="rId58" xr:uid="{EA1DCE00-6252-4B38-B38B-CC6F401BD05B}"/>
+    <hyperlink ref="A20" r:id="rId59" xr:uid="{74330122-414A-4EE6-B7D1-633978CAFC7F}"/>
+    <hyperlink ref="A18" r:id="rId60" xr:uid="{646431EC-C544-4C5B-9C8B-33FA5C080A5B}"/>
+    <hyperlink ref="A17" r:id="rId61" xr:uid="{7AED7DC4-C836-4A03-A289-3731E38BA141}"/>
+    <hyperlink ref="A16" r:id="rId62" xr:uid="{F02129EB-2BBD-443E-9D69-6623A732C49F}"/>
+    <hyperlink ref="A15" r:id="rId63" xr:uid="{424CD5D2-5B3D-46A5-8723-D7AEB663A399}"/>
+    <hyperlink ref="A14" r:id="rId64" xr:uid="{55EF3F12-9C12-468F-B2F7-48B4187B239A}"/>
+    <hyperlink ref="A13" r:id="rId65" xr:uid="{DC84D70E-A9B3-4945-AF4F-0D220AD052C1}"/>
+    <hyperlink ref="A12" r:id="rId66" xr:uid="{680F938F-34DD-4AB6-99C0-A237DBA25C40}"/>
+    <hyperlink ref="A10" r:id="rId67" xr:uid="{F3B2B3FC-3652-463F-AC4B-24093389FED6}"/>
+    <hyperlink ref="A9" r:id="rId68" xr:uid="{52FFDFB6-8BA7-440C-AB0A-C2CC4D263F1D}"/>
+    <hyperlink ref="A8" r:id="rId69" xr:uid="{0B717454-34EB-457E-81FA-5F083E19D92F}"/>
+    <hyperlink ref="A7" r:id="rId70" xr:uid="{79193D90-FBAC-42CF-884B-1B287D33D289}"/>
+    <hyperlink ref="A6" r:id="rId71" xr:uid="{D2388750-EFD9-405D-86AE-BCE3CA89E04B}"/>
+    <hyperlink ref="A5" r:id="rId72" xr:uid="{BAED895C-B388-419D-AA42-EAC5180A469B}"/>
+    <hyperlink ref="A4" r:id="rId73" xr:uid="{444CE840-7C67-4021-86DD-17B2E2040CE2}"/>
+    <hyperlink ref="A3" r:id="rId74" xr:uid="{C46F5ED2-A800-437B-9907-79AB5BC3088C}"/>
+    <hyperlink ref="A2" r:id="rId75" xr:uid="{6A0E4EEF-6185-474B-8E18-1E72C0181781}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId78"/>
+  <pageSetup orientation="portrait" r:id="rId76"/>
   <tableParts count="1">
-    <tablePart r:id="rId79"/>
+    <tablePart r:id="rId77"/>
   </tableParts>
 </worksheet>
 </file>
@@ -6896,157 +6959,157 @@
     <col min="5" max="5" width="16.5703125" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="9" t="s">
+    <row r="1" spans="1:5" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="8" t="s">
         <v>73</v>
       </c>
-      <c r="B1" s="10" t="s">
+      <c r="B1" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="C1" s="10" t="s">
+      <c r="C1" s="9" t="s">
         <v>111</v>
       </c>
-      <c r="D1" s="10" t="s">
+      <c r="D1" s="9" t="s">
         <v>74</v>
       </c>
-      <c r="E1" s="10" t="s">
+      <c r="E1" s="9" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>487</v>
+        <v>485</v>
       </c>
       <c r="B2" s="5">
         <v>1</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="D2" s="5" t="s">
         <v>4</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>489</v>
+        <v>487</v>
       </c>
       <c r="B3" s="5">
         <v>1</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="D3" s="5" t="s">
         <v>4</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>490</v>
+        <v>488</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>491</v>
+        <v>489</v>
       </c>
       <c r="B4" s="5">
         <v>1</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="D4" s="5" t="s">
         <v>4</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>492</v>
+        <v>490</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>493</v>
+        <v>491</v>
       </c>
       <c r="B5" s="5">
         <v>1</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="D5" s="5" t="s">
         <v>4</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>494</v>
+        <v>492</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>495</v>
+        <v>493</v>
       </c>
       <c r="B6" s="5">
         <v>1</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="D6" s="5" t="s">
         <v>4</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>496</v>
+        <v>494</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>497</v>
+        <v>495</v>
       </c>
       <c r="B7" s="5">
         <v>1</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="D7" s="5" t="s">
         <v>4</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>498</v>
+        <v>496</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>499</v>
+        <v>497</v>
       </c>
       <c r="B8" s="5">
         <v>1</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="D8" s="5" t="s">
         <v>4</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>500</v>
+        <v>498</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>501</v>
+        <v>499</v>
       </c>
       <c r="B9" s="5">
         <v>1</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="D9" s="5" t="s">
         <v>4</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>502</v>
+        <v>500</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
@@ -7136,7 +7199,7 @@
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
-        <v>433</v>
+        <v>431</v>
       </c>
       <c r="B15" s="5">
         <v>1</v>
@@ -7148,12 +7211,12 @@
         <v>4</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>434</v>
+        <v>432</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
-        <v>503</v>
+        <v>501</v>
       </c>
       <c r="B16" s="5">
         <v>1</v>
@@ -7165,12 +7228,12 @@
         <v>4</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>504</v>
+        <v>502</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
-        <v>506</v>
+        <v>504</v>
       </c>
       <c r="B17" s="5">
         <v>1</v>
@@ -7185,7 +7248,7 @@
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
-        <v>507</v>
+        <v>505</v>
       </c>
       <c r="B18" s="5">
         <v>1</v>
@@ -7202,7 +7265,7 @@
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
-        <v>513</v>
+        <v>511</v>
       </c>
       <c r="B19" s="5">
         <v>1</v>
@@ -7214,18 +7277,18 @@
         <v>4</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>514</v>
+        <v>512</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
+        <v>412</v>
+      </c>
+      <c r="B20" s="5">
+        <v>1</v>
+      </c>
+      <c r="C20" s="5" t="s">
         <v>413</v>
-      </c>
-      <c r="B20" s="5">
-        <v>1</v>
-      </c>
-      <c r="C20" s="5" t="s">
-        <v>414</v>
       </c>
       <c r="D20" s="5" t="s">
         <v>2</v>
@@ -7234,30 +7297,30 @@
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
       <c r="B21" s="5">
         <v>1</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="D21" s="5" t="s">
         <v>2</v>
       </c>
       <c r="E21" s="7" t="s">
-        <v>480</v>
+        <v>478</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
-        <v>481</v>
+        <v>479</v>
       </c>
       <c r="B22" s="5">
         <v>1</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="D22" s="5" t="s">
         <v>2</v>
@@ -7266,13 +7329,13 @@
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
-        <v>482</v>
+        <v>480</v>
       </c>
       <c r="B23" s="5">
         <v>1</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="D23" s="5" t="s">
         <v>2</v>
@@ -7281,13 +7344,13 @@
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
-        <v>483</v>
+        <v>481</v>
       </c>
       <c r="B24" s="5">
         <v>1</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="D24" s="5" t="s">
         <v>2</v>
@@ -7296,30 +7359,30 @@
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
-        <v>484</v>
+        <v>482</v>
       </c>
       <c r="B25" s="5">
         <v>1</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="D25" s="5" t="s">
         <v>2</v>
       </c>
       <c r="E25" s="5" t="s">
-        <v>485</v>
+        <v>483</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="3" t="s">
-        <v>486</v>
+        <v>484</v>
       </c>
       <c r="B26" s="5">
         <v>1</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="D26" s="5" t="s">
         <v>2</v>
@@ -7328,7 +7391,7 @@
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
-        <v>505</v>
+        <v>503</v>
       </c>
       <c r="B27" s="5">
         <v>1</v>
@@ -7343,7 +7406,7 @@
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="3" t="s">
-        <v>508</v>
+        <v>506</v>
       </c>
       <c r="B28" s="5">
         <v>1</v>
@@ -7358,7 +7421,7 @@
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
-        <v>509</v>
+        <v>507</v>
       </c>
       <c r="B29" s="5">
         <v>1</v>
@@ -7373,7 +7436,7 @@
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" s="3" t="s">
-        <v>510</v>
+        <v>508</v>
       </c>
       <c r="B30" s="5">
         <v>1</v>
@@ -7385,12 +7448,12 @@
         <v>2</v>
       </c>
       <c r="E30" s="5" t="s">
-        <v>511</v>
+        <v>509</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
-        <v>515</v>
+        <v>513</v>
       </c>
       <c r="B31" s="5">
         <v>1</v>
@@ -7455,20 +7518,20 @@
     <col min="5" max="5" width="18.5703125" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="9" t="s">
+    <row r="1" spans="1:5" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="8" t="s">
         <v>73</v>
       </c>
-      <c r="B1" s="10" t="s">
+      <c r="B1" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="C1" s="10" t="s">
+      <c r="C1" s="9" t="s">
         <v>111</v>
       </c>
-      <c r="D1" s="10" t="s">
+      <c r="D1" s="9" t="s">
         <v>74</v>
       </c>
-      <c r="E1" s="10" t="s">
+      <c r="E1" s="9" t="s">
         <v>75</v>
       </c>
     </row>
@@ -7480,7 +7543,7 @@
         <v>1</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>519</v>
+        <v>517</v>
       </c>
       <c r="D2" s="5" t="s">
         <v>4</v>
@@ -7497,7 +7560,7 @@
         <v>1</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>519</v>
+        <v>517</v>
       </c>
       <c r="D3" s="5" t="s">
         <v>4</v>
@@ -7514,7 +7577,7 @@
         <v>1</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>516</v>
+        <v>514</v>
       </c>
       <c r="D4" s="5" t="s">
         <v>4</v>
@@ -7531,7 +7594,7 @@
         <v>1</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>516</v>
+        <v>514</v>
       </c>
       <c r="D5" s="5" t="s">
         <v>4</v>
@@ -7548,7 +7611,7 @@
         <v>1</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>516</v>
+        <v>514</v>
       </c>
       <c r="D6" s="5" t="s">
         <v>4</v>
@@ -7565,7 +7628,7 @@
         <v>1</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>516</v>
+        <v>514</v>
       </c>
       <c r="D7" s="5" t="s">
         <v>4</v>
@@ -7582,7 +7645,7 @@
         <v>1</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>516</v>
+        <v>514</v>
       </c>
       <c r="D8" s="5" t="s">
         <v>4</v>
@@ -7599,7 +7662,7 @@
         <v>1</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>516</v>
+        <v>514</v>
       </c>
       <c r="D9" s="5" t="s">
         <v>4</v>
@@ -7616,7 +7679,7 @@
         <v>1</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>516</v>
+        <v>514</v>
       </c>
       <c r="D10" s="5" t="s">
         <v>4</v>
@@ -7633,7 +7696,7 @@
         <v>1</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>516</v>
+        <v>514</v>
       </c>
       <c r="D11" s="5" t="s">
         <v>4</v>
@@ -7650,7 +7713,7 @@
         <v>1</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>516</v>
+        <v>514</v>
       </c>
       <c r="D12" s="5" t="s">
         <v>4</v>
@@ -7667,7 +7730,7 @@
         <v>1</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>516</v>
+        <v>514</v>
       </c>
       <c r="D13" s="5" t="s">
         <v>4</v>
@@ -7684,7 +7747,7 @@
         <v>1</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>516</v>
+        <v>514</v>
       </c>
       <c r="D14" s="5" t="s">
         <v>4</v>
@@ -7701,7 +7764,7 @@
         <v>1</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>516</v>
+        <v>514</v>
       </c>
       <c r="D15" s="5" t="s">
         <v>4</v>
@@ -7718,7 +7781,7 @@
         <v>1</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>516</v>
+        <v>514</v>
       </c>
       <c r="D16" s="5" t="s">
         <v>4</v>
@@ -7735,7 +7798,7 @@
         <v>1</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>516</v>
+        <v>514</v>
       </c>
       <c r="D17" s="5" t="s">
         <v>4</v>
@@ -7752,7 +7815,7 @@
         <v>1</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>516</v>
+        <v>514</v>
       </c>
       <c r="D18" s="5" t="s">
         <v>4</v>
@@ -7769,7 +7832,7 @@
         <v>1</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>516</v>
+        <v>514</v>
       </c>
       <c r="D19" s="5" t="s">
         <v>4</v>
@@ -7786,7 +7849,7 @@
         <v>1</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>516</v>
+        <v>514</v>
       </c>
       <c r="D20" s="5" t="s">
         <v>4</v>
@@ -7803,7 +7866,7 @@
         <v>1</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>516</v>
+        <v>514</v>
       </c>
       <c r="D21" s="5" t="s">
         <v>4</v>
@@ -7820,7 +7883,7 @@
         <v>1</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>516</v>
+        <v>514</v>
       </c>
       <c r="D22" s="5" t="s">
         <v>4</v>
@@ -7837,7 +7900,7 @@
         <v>1</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>516</v>
+        <v>514</v>
       </c>
       <c r="D23" s="5" t="s">
         <v>4</v>
@@ -7854,7 +7917,7 @@
         <v>1</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>516</v>
+        <v>514</v>
       </c>
       <c r="D24" s="5" t="s">
         <v>4</v>
@@ -7871,7 +7934,7 @@
         <v>1</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>516</v>
+        <v>514</v>
       </c>
       <c r="D25" s="5" t="s">
         <v>4</v>
@@ -7888,7 +7951,7 @@
         <v>1</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>516</v>
+        <v>514</v>
       </c>
       <c r="D26" s="5" t="s">
         <v>4</v>
@@ -7905,7 +7968,7 @@
         <v>1</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>516</v>
+        <v>514</v>
       </c>
       <c r="D27" s="5" t="s">
         <v>4</v>
@@ -7922,7 +7985,7 @@
         <v>1</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>516</v>
+        <v>514</v>
       </c>
       <c r="D28" s="5" t="s">
         <v>4</v>
@@ -7933,13 +7996,13 @@
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
-        <v>444</v>
+        <v>442</v>
       </c>
       <c r="B29" s="5">
         <v>1</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>516</v>
+        <v>514</v>
       </c>
       <c r="D29" s="5" t="s">
         <v>4</v>
@@ -7954,7 +8017,7 @@
         <v>1</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>519</v>
+        <v>517</v>
       </c>
       <c r="D30" s="5" t="s">
         <v>2</v>
@@ -7965,30 +8028,30 @@
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
+        <v>515</v>
+      </c>
+      <c r="B31" s="5">
+        <v>1</v>
+      </c>
+      <c r="C31" s="5" t="s">
         <v>517</v>
       </c>
-      <c r="B31" s="5">
-        <v>1</v>
-      </c>
-      <c r="C31" s="5" t="s">
-        <v>519</v>
-      </c>
       <c r="D31" s="5" t="s">
         <v>2</v>
       </c>
       <c r="E31" s="5" t="s">
-        <v>518</v>
+        <v>516</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" s="3" t="s">
-        <v>445</v>
+        <v>443</v>
       </c>
       <c r="B32" s="5">
         <v>1</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>521</v>
+        <v>519</v>
       </c>
       <c r="D32" s="5" t="s">
         <v>2</v>
@@ -8003,7 +8066,7 @@
         <v>1</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>516</v>
+        <v>514</v>
       </c>
       <c r="D33" s="5" t="s">
         <v>2</v>
@@ -8012,13 +8075,13 @@
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" s="3" t="s">
-        <v>442</v>
+        <v>440</v>
       </c>
       <c r="B34" s="5">
         <v>1</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>516</v>
+        <v>514</v>
       </c>
       <c r="D34" s="5" t="s">
         <v>2</v>
@@ -8027,13 +8090,13 @@
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" s="3" t="s">
-        <v>443</v>
+        <v>441</v>
       </c>
       <c r="B35" s="5">
         <v>1</v>
       </c>
       <c r="C35" s="5" t="s">
-        <v>520</v>
+        <v>518</v>
       </c>
       <c r="D35" s="5" t="s">
         <v>2</v>

</xml_diff>